<commit_message>
Updated BRA_grids model - 2025-09-09 19:50
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{033808B8-8A19-4E73-B247-5809D0614E13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C9121CAE-5C36-4702-B995-1754C5BEC885}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22001,7 +22001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8F8293A-8A14-414C-8BA1-65972DD02A92}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44819861-42F3-4A24-A9D1-F43700F568CC}">
   <dimension ref="B9:E3479"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-09 21:07
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C9121CAE-5C36-4702-B995-1754C5BEC885}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3B18C535-CD7F-4F27-A223-75A005D30D23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22001,7 +22001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44819861-42F3-4A24-A9D1-F43700F568CC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4AEB857-B009-4239-A488-4A614905572D}">
   <dimension ref="B9:E3479"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-09 23:29
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3B18C535-CD7F-4F27-A223-75A005D30D23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{119401AF-4A8C-42FF-97CA-D4FF3162BA20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22001,7 +22001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4AEB857-B009-4239-A488-4A614905572D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{561DF167-CD2D-470D-AF82-5083A740B6F2}">
   <dimension ref="B9:E3479"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-11 19:40
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0DC5636C-C62A-48CB-B277-3FE93C2E07F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9AF124CC-05FE-42F6-8DDE-05A8F60DE6C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22001,7 +22001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9397B95-A786-417D-A3EA-11F101A7AE6B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F19D85B2-796D-424A-9C5A-719F45E22B1D}">
   <dimension ref="B9:E3479"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-14 13:59
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9AF124CC-05FE-42F6-8DDE-05A8F60DE6C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DE3040F6-1227-49A6-AFA7-67D29E2496A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22001,7 +22001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F19D85B2-796D-424A-9C5A-719F45E22B1D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7212C178-9807-45CF-9484-D58A04BADE45}">
   <dimension ref="B9:E3479"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-17 01:24
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DE3040F6-1227-49A6-AFA7-67D29E2496A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1D51409E-EA2E-4992-8DB5-9009100D289F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1103" yWindow="1103" windowWidth="21600" windowHeight="12682" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
@@ -22001,7 +22001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7212C178-9807-45CF-9484-D58A04BADE45}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{896FA6B6-A68F-4CD4-98A4-89099C20CAE2}">
   <dimension ref="B9:E3479"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-17 02:24
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1D51409E-EA2E-4992-8DB5-9009100D289F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C3290E1-0751-4798-97DE-82F7EC3E5C08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1103" yWindow="1103" windowWidth="21600" windowHeight="12682" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2573" yWindow="2573" windowWidth="21600" windowHeight="12682" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
@@ -22001,7 +22001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{896FA6B6-A68F-4CD4-98A4-89099C20CAE2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{045961B5-8C89-475C-96B8-C9E11F9019EE}">
   <dimension ref="B9:E3479"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-17 09:49
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C3290E1-0751-4798-97DE-82F7EC3E5C08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3F988052-AF58-4D1D-A987-3B2F5AC06CB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2573" yWindow="2573" windowWidth="21600" windowHeight="12682" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
@@ -22001,7 +22001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{045961B5-8C89-475C-96B8-C9E11F9019EE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8930446D-8A98-45E9-A8D8-66A90C598415}">
   <dimension ref="B9:E3479"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-21 00:19
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5726E500-633C-42D5-B60A-BEA6C72A256A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{891BF29E-7B8A-4610-8B95-BA2AE6EBBA98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4403,7 +4403,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49EE7463-8442-4C0F-B500-89CCA348612B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{030EB6CF-CC52-46FA-812D-CF9F035137D8}">
   <dimension ref="B9:E546"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-22 23:14
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DD796B44-22DD-45B8-9E0A-1E3D662BBEB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A724DAD6-ABC2-48CB-A455-EFF13F3D8D39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4403,7 +4403,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F67B3097-0E1D-4D50-9694-9FF2128C1B22}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4295882D-9480-4B1C-AE21-1DE159C975D5}">
   <dimension ref="B9:E546"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-26 22:16
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8547E82E-1BFB-4057-9F96-BDB61E065033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F6561E6E-C455-47B3-8D82-40D0EB5A245C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4403,7 +4403,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70E063FB-4568-42F1-B4FE-4833416D3FE8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F7D564D-C443-4A9B-8140-E02BADA19D9D}">
   <dimension ref="B9:E546"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>